<commit_message>
Fix theoretical IPO returns using day1/day2 high-low range
Store first- and second-day high/low for each listing, redefine
theory max as buy day1 low / sell day2 high, and render a dashed
range bar against actual trade yield.

Co-authored-by: maoyimin2007 <maoyimin2007@gmail.com>
</commit_message>
<xml_diff>
--- a/data/2026新股_按上市日期.xlsx
+++ b/data/2026新股_按上市日期.xlsx
@@ -11,7 +11,7 @@
     <sheet name="字段说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026新股'!$A$3:$AB$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026新股'!$A$3:$AG$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB59"/>
+  <dimension ref="A1:AG59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -718,25 +718,50 @@
       </c>
       <c r="X3" s="3" t="inlineStr">
         <is>
+          <t>首日最高价(元)</t>
+        </is>
+      </c>
+      <c r="Y3" s="3" t="inlineStr">
+        <is>
+          <t>首日最低价(元)</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
+          <t>次日日期</t>
+        </is>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>次日最高价(元)</t>
+        </is>
+      </c>
+      <c r="AB3" s="3" t="inlineStr">
+        <is>
+          <t>次日最低价(元)</t>
+        </is>
+      </c>
+      <c r="AC3" s="3" t="inlineStr">
+        <is>
           <t>首日涨跌幅(%)</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
+      <c r="AD3" s="3" t="inlineStr">
         <is>
           <t>发行市盈率</t>
         </is>
       </c>
-      <c r="Z3" s="3" t="inlineStr">
+      <c r="AE3" s="3" t="inlineStr">
         <is>
           <t>保荐机构</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AF3" s="3" t="inlineStr">
         <is>
           <t>主营业务</t>
         </is>
       </c>
-      <c r="AB3" s="3" t="inlineStr">
+      <c r="AG3" s="3" t="inlineStr">
         <is>
           <t>公司全称</t>
         </is>
@@ -829,22 +854,39 @@
         <v>132</v>
       </c>
       <c r="X4" s="6" t="n">
+        <v>152</v>
+      </c>
+      <c r="Y4" s="6" t="n">
+        <v>125</v>
+      </c>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="AA4" s="6" t="n">
+        <v>147.39</v>
+      </c>
+      <c r="AB4" s="6" t="n">
+        <v>134</v>
+      </c>
+      <c r="AC4" s="6" t="n">
         <v>64.09999999999999</v>
       </c>
-      <c r="Y4" s="6" t="n">
+      <c r="AD4" s="6" t="n">
         <v>12.37</v>
       </c>
-      <c r="Z4" s="5" t="inlineStr">
+      <c r="AE4" s="5" t="inlineStr">
         <is>
           <t>中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA4" s="5" t="inlineStr">
+      <c r="AF4" s="5" t="inlineStr">
         <is>
           <t>集旅游演艺、旅游索道、旅游餐饮、旅游项目投资及管理为一体,依托华清宫、华山等优质旅游资源,充分发挥旅游资源整合优势、专业化运营管理优势、旅游产品创新优势,为游客提供高品质的旅游产品及服务体验</t>
         </is>
       </c>
-      <c r="AB4" s="5" t="inlineStr">
+      <c r="AG4" s="5" t="inlineStr">
         <is>
           <t>陕西旅游文化产业股份有限公司</t>
         </is>
@@ -937,22 +979,39 @@
         <v>68.58</v>
       </c>
       <c r="X5" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="Y5" s="11" t="n">
+        <v>66</v>
+      </c>
+      <c r="Z5" s="10" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="AA5" s="11" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="AB5" s="11" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="AC5" s="11" t="n">
         <v>213.44</v>
       </c>
-      <c r="Y5" s="11" t="n">
+      <c r="AD5" s="11" t="n">
         <v>26.85</v>
       </c>
-      <c r="Z5" s="10" t="inlineStr">
+      <c r="AE5" s="10" t="inlineStr">
         <is>
           <t>申万宏源证券承销保荐有限责任公司</t>
         </is>
       </c>
-      <c r="AA5" s="10" t="inlineStr">
+      <c r="AF5" s="10" t="inlineStr">
         <is>
           <t>汽车冲焊件以及相关模具的开发、加工、生产和销售</t>
         </is>
       </c>
-      <c r="AB5" s="10" t="inlineStr">
+      <c r="AG5" s="10" t="inlineStr">
         <is>
           <t>重庆至信实业股份有限公司</t>
         </is>
@@ -1045,22 +1104,39 @@
         <v>371.3</v>
       </c>
       <c r="X6" s="6" t="n">
+        <v>390</v>
+      </c>
+      <c r="Y6" s="6" t="n">
+        <v>310</v>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="AA6" s="6" t="n">
+        <v>421</v>
+      </c>
+      <c r="AB6" s="6" t="n">
+        <v>340</v>
+      </c>
+      <c r="AC6" s="6" t="n">
         <v>302.8</v>
       </c>
-      <c r="Y6" s="6" t="n">
+      <c r="AD6" s="6" t="n">
         <v>48.39</v>
       </c>
-      <c r="Z6" s="5" t="inlineStr">
+      <c r="AE6" s="5" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA6" s="5" t="inlineStr">
+      <c r="AF6" s="5" t="inlineStr">
         <is>
           <t>等离子体射频电源系统、等离子体激发装置、等离子体直流电源、各种配件的研发、生产、销售及技术服务,并引进真空获得和流体控制等相关的核心零部件,围绕等离子体工艺提供核心零部件整体解决方案</t>
         </is>
       </c>
-      <c r="AB6" s="5" t="inlineStr">
+      <c r="AG6" s="5" t="inlineStr">
         <is>
           <t>深圳市恒运昌真空技术股份有限公司</t>
         </is>
@@ -1153,22 +1229,39 @@
         <v>24.78</v>
       </c>
       <c r="X7" s="11" t="n">
+        <v>31</v>
+      </c>
+      <c r="Y7" s="11" t="n">
+        <v>24.31</v>
+      </c>
+      <c r="Z7" s="10" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="AA7" s="11" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="AB7" s="11" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="AC7" s="11" t="n">
         <v>121.65</v>
       </c>
-      <c r="Y7" s="11" t="n">
+      <c r="AD7" s="11" t="n">
         <v>32.59</v>
       </c>
-      <c r="Z7" s="10" t="inlineStr">
+      <c r="AE7" s="10" t="inlineStr">
         <is>
           <t>中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA7" s="10" t="inlineStr">
+      <c r="AF7" s="10" t="inlineStr">
         <is>
           <t>清洁能源领域纤维增强材料研发、生产及销售</t>
         </is>
       </c>
-      <c r="AB7" s="10" t="inlineStr">
+      <c r="AG7" s="10" t="inlineStr">
         <is>
           <t>浙江振石新材料股份有限公司</t>
         </is>
@@ -1261,22 +1354,39 @@
         <v>57.73</v>
       </c>
       <c r="X8" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="Y8" s="6" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="Z8" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="AA8" s="6" t="n">
+        <v>55.68</v>
+      </c>
+      <c r="AB8" s="6" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="AC8" s="6" t="n">
         <v>106.18</v>
       </c>
-      <c r="Y8" s="6" t="n">
+      <c r="AD8" s="6" t="n">
         <v>15.29</v>
       </c>
-      <c r="Z8" s="5" t="inlineStr">
+      <c r="AE8" s="5" t="inlineStr">
         <is>
           <t>中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA8" s="5" t="inlineStr">
+      <c r="AF8" s="5" t="inlineStr">
         <is>
           <t>为跨国制造企业提供定制化、一体化、嵌入式的供应链物流解决方案</t>
         </is>
       </c>
-      <c r="AB8" s="5" t="inlineStr">
+      <c r="AG8" s="5" t="inlineStr">
         <is>
           <t>世盟供应链管理股份有限公司</t>
         </is>
@@ -1369,20 +1479,37 @@
         <v>49.64</v>
       </c>
       <c r="X9" s="11" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="Y9" s="11" t="n">
+        <v>47</v>
+      </c>
+      <c r="Z9" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="AA9" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="AB9" s="11" t="n">
+        <v>47</v>
+      </c>
+      <c r="AC9" s="11" t="n">
         <v>183.33</v>
       </c>
-      <c r="Y9" s="10" t="n"/>
-      <c r="Z9" s="10" t="inlineStr">
+      <c r="AD9" s="10" t="n"/>
+      <c r="AE9" s="10" t="inlineStr">
         <is>
           <t>中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA9" s="10" t="inlineStr">
+      <c r="AF9" s="10" t="inlineStr">
         <is>
           <t>专注于心血管疾病精准介入解决方案的医疗科技企业,自2015年成立以来,始终秉持并笃行“用创新和品质改善生命健康”的使命,致力于为冠状动脉疾病、外周血管疾病及心律失常等严重影响生命健康的心血管疾病提供创新智能化精准介入解决方案,持续助力临床提升诊疗水平。</t>
         </is>
       </c>
-      <c r="AB9" s="10" t="inlineStr">
+      <c r="AG9" s="10" t="inlineStr">
         <is>
           <t>深圳北芯生命科技股份有限公司</t>
         </is>
@@ -1475,22 +1602,39 @@
         <v>58.93</v>
       </c>
       <c r="X10" s="6" t="n">
+        <v>75.13</v>
+      </c>
+      <c r="Y10" s="6" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="Z10" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="AA10" s="6" t="n">
+        <v>55.96</v>
+      </c>
+      <c r="AB10" s="6" t="n">
+        <v>52.22</v>
+      </c>
+      <c r="AC10" s="6" t="n">
         <v>55.57</v>
       </c>
-      <c r="Y10" s="6" t="n">
+      <c r="AD10" s="6" t="n">
         <v>18.69</v>
       </c>
-      <c r="Z10" s="5" t="inlineStr">
+      <c r="AE10" s="5" t="inlineStr">
         <is>
           <t>国联民生证券承销保荐有限公司</t>
         </is>
       </c>
-      <c r="AA10" s="5" t="inlineStr">
+      <c r="AF10" s="5" t="inlineStr">
         <is>
           <t>包装用原纸产品的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB10" s="5" t="inlineStr">
+      <c r="AG10" s="5" t="inlineStr">
         <is>
           <t>安徽林平循环发展股份有限公司</t>
         </is>
@@ -1583,22 +1727,39 @@
         <v>65.94</v>
       </c>
       <c r="X11" s="11" t="n">
+        <v>80.88</v>
+      </c>
+      <c r="Y11" s="11" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="Z11" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="AA11" s="11" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="AB11" s="11" t="n">
+        <v>62.06</v>
+      </c>
+      <c r="AC11" s="11" t="n">
         <v>596.3</v>
       </c>
-      <c r="Y11" s="11" t="n">
+      <c r="AD11" s="11" t="n">
         <v>56.79</v>
       </c>
-      <c r="Z11" s="10" t="inlineStr">
+      <c r="AE11" s="10" t="inlineStr">
         <is>
           <t>中信建投证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA11" s="10" t="inlineStr">
+      <c r="AF11" s="10" t="inlineStr">
         <is>
           <t>电能源产品及系统的研发、生产、销售及服务</t>
         </is>
       </c>
-      <c r="AB11" s="10" t="inlineStr">
+      <c r="AG11" s="10" t="inlineStr">
         <is>
           <t>中电科蓝天科技股份有限公司</t>
         </is>
@@ -1691,22 +1852,39 @@
         <v>88.92</v>
       </c>
       <c r="X12" s="6" t="n">
+        <v>107.98</v>
+      </c>
+      <c r="Y12" s="6" t="n">
+        <v>86</v>
+      </c>
+      <c r="Z12" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="AA12" s="6" t="n">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="AB12" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="AC12" s="6" t="n">
         <v>58.93</v>
       </c>
-      <c r="Y12" s="6" t="n">
+      <c r="AD12" s="6" t="n">
         <v>90.39</v>
       </c>
-      <c r="Z12" s="5" t="inlineStr">
+      <c r="AE12" s="5" t="inlineStr">
         <is>
           <t>国投证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA12" s="5" t="inlineStr">
+      <c r="AF12" s="5" t="inlineStr">
         <is>
           <t>汽车制造机器视觉设备的研发、生产及销售</t>
         </is>
       </c>
-      <c r="AB12" s="5" t="inlineStr">
+      <c r="AG12" s="5" t="inlineStr">
         <is>
           <t>易思维(杭州)科技股份有限公司</t>
         </is>
@@ -1799,22 +1977,39 @@
         <v>126.71</v>
       </c>
       <c r="X13" s="11" t="n">
+        <v>147.82</v>
+      </c>
+      <c r="Y13" s="11" t="n">
+        <v>125</v>
+      </c>
+      <c r="Z13" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="AA13" s="11" t="n">
+        <v>128.9</v>
+      </c>
+      <c r="AB13" s="11" t="n">
+        <v>113.8</v>
+      </c>
+      <c r="AC13" s="11" t="n">
         <v>118.47</v>
       </c>
-      <c r="Y13" s="11" t="n">
+      <c r="AD13" s="11" t="n">
         <v>27.96</v>
       </c>
-      <c r="Z13" s="10" t="inlineStr">
+      <c r="AE13" s="10" t="inlineStr">
         <is>
           <t>东吴证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA13" s="10" t="inlineStr">
+      <c r="AF13" s="10" t="inlineStr">
         <is>
           <t>新能源汽车动力电池热失控防护零部件及电力电工绝缘产品的研发、生产和销售,为客户提供定制化的热失控防护解决方案和电力电工高性能绝缘解决方案</t>
         </is>
       </c>
-      <c r="AB13" s="10" t="inlineStr">
+      <c r="AG13" s="10" t="inlineStr">
         <is>
           <t>固德电材系统(苏州)股份有限公司</t>
         </is>
@@ -1907,22 +2102,39 @@
         <v>128.65</v>
       </c>
       <c r="X14" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="Y14" s="6" t="n">
+        <v>128</v>
+      </c>
+      <c r="Z14" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="AA14" s="6" t="n">
+        <v>136.68</v>
+      </c>
+      <c r="AB14" s="6" t="n">
+        <v>128.88</v>
+      </c>
+      <c r="AC14" s="6" t="n">
         <v>84.68000000000001</v>
       </c>
-      <c r="Y14" s="6" t="n">
+      <c r="AD14" s="6" t="n">
         <v>33.61</v>
       </c>
-      <c r="Z14" s="5" t="inlineStr">
+      <c r="AE14" s="5" t="inlineStr">
         <is>
           <t>申万宏源证券承销保荐有限责任公司</t>
         </is>
       </c>
-      <c r="AA14" s="5" t="inlineStr">
+      <c r="AF14" s="5" t="inlineStr">
         <is>
           <t>以阻容元器件为主的新型电子元器件及精密零组件的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB14" s="5" t="inlineStr">
+      <c r="AG14" s="5" t="inlineStr">
         <is>
           <t>成都宏明电子股份有限公司</t>
         </is>
@@ -2015,20 +2227,37 @@
         <v>46</v>
       </c>
       <c r="X15" s="11" t="n">
+        <v>52.88</v>
+      </c>
+      <c r="Y15" s="11" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="Z15" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="AA15" s="11" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="AB15" s="11" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="AC15" s="11" t="n">
         <v>102.82</v>
       </c>
-      <c r="Y15" s="10" t="n"/>
-      <c r="Z15" s="10" t="inlineStr">
+      <c r="AD15" s="10" t="n"/>
+      <c r="AE15" s="10" t="inlineStr">
         <is>
           <t>国泰海通证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA15" s="10" t="inlineStr">
+      <c r="AF15" s="10" t="inlineStr">
         <is>
           <t>硅基OLED微型显示屏、光学系统和XR整体解决方案的研发、生产制造和销售、战略产品开发</t>
         </is>
       </c>
-      <c r="AB15" s="10" t="inlineStr">
+      <c r="AG15" s="10" t="inlineStr">
         <is>
           <t>视涯科技股份有限公司</t>
         </is>
@@ -2121,22 +2350,39 @@
         <v>27.68</v>
       </c>
       <c r="X16" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y16" s="6" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="Z16" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="AA16" s="6" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="AB16" s="6" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="AC16" s="6" t="n">
         <v>253.96</v>
       </c>
-      <c r="Y16" s="6" t="n">
+      <c r="AD16" s="6" t="n">
         <v>19.11</v>
       </c>
-      <c r="Z16" s="5" t="inlineStr">
+      <c r="AE16" s="5" t="inlineStr">
         <is>
           <t>国投证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA16" s="5" t="inlineStr">
+      <c r="AF16" s="5" t="inlineStr">
         <is>
           <t>钼相关产品的生产、加工、销售业务</t>
         </is>
       </c>
-      <c r="AB16" s="5" t="inlineStr">
+      <c r="AG16" s="5" t="inlineStr">
         <is>
           <t>洛阳盛龙矿业集团股份有限公司</t>
         </is>
@@ -2229,22 +2475,39 @@
         <v>49.47</v>
       </c>
       <c r="X17" s="11" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="Y17" s="11" t="n">
+        <v>47.01</v>
+      </c>
+      <c r="Z17" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="AA17" s="11" t="n">
+        <v>52.77</v>
+      </c>
+      <c r="AB17" s="11" t="n">
+        <v>46.61</v>
+      </c>
+      <c r="AC17" s="11" t="n">
         <v>88.23999999999999</v>
       </c>
-      <c r="Y17" s="11" t="n">
+      <c r="AD17" s="11" t="n">
         <v>22.94</v>
       </c>
-      <c r="Z17" s="10" t="inlineStr">
+      <c r="AE17" s="10" t="inlineStr">
         <is>
           <t>中信建投证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA17" s="10" t="inlineStr">
+      <c r="AF17" s="10" t="inlineStr">
         <is>
           <t>专注于高端绿色电解成套装备、钛电极以及金属玻璃封接制品的研发、设计、生产及销售</t>
         </is>
       </c>
-      <c r="AB17" s="10" t="inlineStr">
+      <c r="AG17" s="10" t="inlineStr">
         <is>
           <t>西安泰金新能科技股份有限公司</t>
         </is>
@@ -2337,22 +2600,39 @@
         <v>126.71</v>
       </c>
       <c r="X18" s="6" t="n">
+        <v>158</v>
+      </c>
+      <c r="Y18" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="Z18" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="AA18" s="6" t="n">
+        <v>133.12</v>
+      </c>
+      <c r="AB18" s="6" t="n">
+        <v>123</v>
+      </c>
+      <c r="AC18" s="6" t="n">
         <v>61.66</v>
       </c>
-      <c r="Y18" s="6" t="n">
+      <c r="AD18" s="6" t="n">
         <v>34.91</v>
       </c>
-      <c r="Z18" s="5" t="inlineStr">
+      <c r="AE18" s="5" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA18" s="5" t="inlineStr">
+      <c r="AF18" s="5" t="inlineStr">
         <is>
           <t>功能性树脂和功能性涂层材料的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB18" s="5" t="inlineStr">
+      <c r="AG18" s="5" t="inlineStr">
         <is>
           <t>广州慧谷新材料科技股份有限公司</t>
         </is>
@@ -2445,22 +2725,39 @@
         <v>57.7</v>
       </c>
       <c r="X19" s="11" t="n">
+        <v>67.59</v>
+      </c>
+      <c r="Y19" s="11" t="n">
+        <v>49</v>
+      </c>
+      <c r="Z19" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="AA19" s="11" t="n">
+        <v>54.44</v>
+      </c>
+      <c r="AB19" s="11" t="n">
+        <v>50.11</v>
+      </c>
+      <c r="AC19" s="11" t="n">
         <v>225.99</v>
       </c>
-      <c r="Y19" s="11" t="n">
+      <c r="AD19" s="11" t="n">
         <v>25.6</v>
       </c>
-      <c r="Z19" s="10" t="inlineStr">
+      <c r="AE19" s="10" t="inlineStr">
         <is>
           <t>国联民生证券承销保荐有限公司</t>
         </is>
       </c>
-      <c r="AA19" s="10" t="inlineStr">
+      <c r="AF19" s="10" t="inlineStr">
         <is>
           <t>公司专注于印制电路板的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB19" s="10" t="inlineStr">
+      <c r="AG19" s="10" t="inlineStr">
         <is>
           <t>江西红板科技股份有限公司</t>
         </is>
@@ -2553,22 +2850,39 @@
         <v>92</v>
       </c>
       <c r="X20" s="6" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="Y20" s="6" t="n">
+        <v>85.73</v>
+      </c>
+      <c r="Z20" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="AA20" s="6" t="n">
+        <v>121</v>
+      </c>
+      <c r="AB20" s="6" t="n">
+        <v>102</v>
+      </c>
+      <c r="AC20" s="6" t="n">
         <v>272.77</v>
       </c>
-      <c r="Y20" s="6" t="n">
+      <c r="AD20" s="6" t="n">
         <v>30.8</v>
       </c>
-      <c r="Z20" s="5" t="inlineStr">
+      <c r="AE20" s="5" t="inlineStr">
         <is>
           <t>国泰海通证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA20" s="5" t="inlineStr">
+      <c r="AF20" s="5" t="inlineStr">
         <is>
           <t>无人机电动动力系统及机器人动力系统的研发、生产和销售,并积极布局电动垂直起降飞行器(eVTOL)动力系统产品</t>
         </is>
       </c>
-      <c r="AB20" s="5" t="inlineStr">
+      <c r="AG20" s="5" t="inlineStr">
         <is>
           <t>南昌三瑞智能科技股份有限公司</t>
         </is>
@@ -2661,22 +2975,39 @@
         <v>17.12</v>
       </c>
       <c r="X21" s="11" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="Y21" s="11" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="Z21" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="AA21" s="11" t="n">
+        <v>18.93</v>
+      </c>
+      <c r="AB21" s="11" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="AC21" s="11" t="n">
         <v>167.08</v>
       </c>
-      <c r="Y21" s="11" t="n">
+      <c r="AD21" s="11" t="n">
         <v>58.09</v>
       </c>
-      <c r="Z21" s="10" t="inlineStr">
+      <c r="AE21" s="10" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA21" s="10" t="inlineStr">
+      <c r="AF21" s="10" t="inlineStr">
         <is>
           <t>金属复合材料及制品、特种有色金属合金制品的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB21" s="10" t="inlineStr">
+      <c r="AG21" s="10" t="inlineStr">
         <is>
           <t>有研金属复合材料(北京)股份公司</t>
         </is>
@@ -2769,20 +3100,37 @@
         <v>244.55</v>
       </c>
       <c r="X22" s="6" t="n">
+        <v>255</v>
+      </c>
+      <c r="Y22" s="6" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="Z22" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="AA22" s="6" t="n">
+        <v>266</v>
+      </c>
+      <c r="AB22" s="6" t="n">
+        <v>229.8</v>
+      </c>
+      <c r="AC22" s="6" t="n">
         <v>430.71</v>
       </c>
-      <c r="Y22" s="5" t="n"/>
-      <c r="Z22" s="5" t="inlineStr">
+      <c r="AD22" s="5" t="n"/>
+      <c r="AE22" s="5" t="inlineStr">
         <is>
           <t>国泰海通证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA22" s="5" t="inlineStr">
+      <c r="AF22" s="5" t="inlineStr">
         <is>
           <t>数据中心企业级SSD产品的研发和销售</t>
         </is>
       </c>
-      <c r="AB22" s="5" t="inlineStr">
+      <c r="AG22" s="5" t="inlineStr">
         <is>
           <t>深圳大普微电子股份有限公司</t>
         </is>
@@ -2875,22 +3223,39 @@
         <v>71.02</v>
       </c>
       <c r="X23" s="11" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="Y23" s="11" t="n">
+        <v>71</v>
+      </c>
+      <c r="Z23" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="AA23" s="11" t="n">
+        <v>68.42</v>
+      </c>
+      <c r="AB23" s="11" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="AC23" s="11" t="n">
         <v>112.06</v>
       </c>
-      <c r="Y23" s="11" t="n">
+      <c r="AD23" s="11" t="n">
         <v>29.71</v>
       </c>
-      <c r="Z23" s="10" t="inlineStr">
+      <c r="AE23" s="10" t="inlineStr">
         <is>
           <t>华泰联合证券有限责任公司</t>
         </is>
       </c>
-      <c r="AA23" s="10" t="inlineStr">
+      <c r="AF23" s="10" t="inlineStr">
         <is>
           <t>从事车身域、智能座舱域、动力域以及智能驾驶域等汽车电子产品的研发、生产及销售,同时为客户提供汽车电子EMS和技术开发服务。</t>
         </is>
       </c>
-      <c r="AB23" s="10" t="inlineStr">
+      <c r="AG23" s="10" t="inlineStr">
         <is>
           <t>芜湖埃泰克汽车电子股份有限公司</t>
         </is>
@@ -2983,22 +3348,39 @@
         <v>103.1</v>
       </c>
       <c r="X24" s="6" t="n">
+        <v>116.78</v>
+      </c>
+      <c r="Y24" s="6" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="Z24" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="AA24" s="6" t="n">
+        <v>99.45</v>
+      </c>
+      <c r="AB24" s="6" t="n">
+        <v>89.01000000000001</v>
+      </c>
+      <c r="AC24" s="6" t="n">
         <v>286.72</v>
       </c>
-      <c r="Y24" s="6" t="n">
+      <c r="AD24" s="6" t="n">
         <v>18.02</v>
       </c>
-      <c r="Z24" s="5" t="inlineStr">
+      <c r="AE24" s="5" t="inlineStr">
         <is>
           <t>国联民生证券承销保荐有限公司</t>
         </is>
       </c>
-      <c r="AA24" s="5" t="inlineStr">
+      <c r="AF24" s="5" t="inlineStr">
         <is>
           <t>围绕微纳粉体处理、粉液精密计量、粉液混合分散、功能薄膜制备等核心工艺环节展开,产品可广泛用于新能源电池、新材料、化工、食品、医药、半导体等行业。目前公司主要面向新能源电池极片制造及新材料制备领域,专业从事融合工艺能力的智能装备的研发、设计、生产与销售</t>
         </is>
       </c>
-      <c r="AB24" s="5" t="inlineStr">
+      <c r="AG24" s="5" t="inlineStr">
         <is>
           <t>深圳市尚水智能股份有限公司</t>
         </is>
@@ -3091,22 +3473,39 @@
         <v>76.65000000000001</v>
       </c>
       <c r="X25" s="11" t="n">
+        <v>100.99</v>
+      </c>
+      <c r="Y25" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z25" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="AA25" s="11" t="n">
+        <v>96.22</v>
+      </c>
+      <c r="AB25" s="11" t="n">
+        <v>75.02</v>
+      </c>
+      <c r="AC25" s="11" t="n">
         <v>289.48</v>
       </c>
-      <c r="Y25" s="11" t="n">
+      <c r="AD25" s="11" t="n">
         <v>195.62</v>
       </c>
-      <c r="Z25" s="10" t="inlineStr">
+      <c r="AE25" s="10" t="inlineStr">
         <is>
           <t>中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA25" s="10" t="inlineStr">
+      <c r="AF25" s="10" t="inlineStr">
         <is>
           <t>中段硅片加工、晶圆级封装、芯粒多芯片集成封装等晶圆级先进封测服务</t>
         </is>
       </c>
-      <c r="AB25" s="10" t="inlineStr">
+      <c r="AG25" s="10" t="inlineStr">
         <is>
           <t>盛合晶微半导体有限公司</t>
         </is>
@@ -3199,22 +3598,39 @@
         <v>30.57</v>
       </c>
       <c r="X26" s="6" t="n">
+        <v>36.53</v>
+      </c>
+      <c r="Y26" s="6" t="n">
+        <v>30.11</v>
+      </c>
+      <c r="Z26" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="AA26" s="6" t="n">
+        <v>30.32</v>
+      </c>
+      <c r="AB26" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="AC26" s="6" t="n">
         <v>66.31999999999999</v>
       </c>
-      <c r="Y26" s="6" t="n">
+      <c r="AD26" s="6" t="n">
         <v>16.83</v>
       </c>
-      <c r="Z26" s="5" t="inlineStr">
+      <c r="AE26" s="5" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA26" s="5" t="inlineStr">
+      <c r="AF26" s="5" t="inlineStr">
         <is>
           <t>从事生态环保面料的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB26" s="5" t="inlineStr">
+      <c r="AG26" s="5" t="inlineStr">
         <is>
           <t>杭州福恩股份有限公司</t>
         </is>
@@ -3307,22 +3723,39 @@
         <v>799</v>
       </c>
       <c r="X27" s="11" t="n">
+        <v>859.88</v>
+      </c>
+      <c r="Y27" s="11" t="n">
+        <v>688.99</v>
+      </c>
+      <c r="Z27" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="AA27" s="11" t="n">
+        <v>900</v>
+      </c>
+      <c r="AB27" s="11" t="n">
+        <v>810.02</v>
+      </c>
+      <c r="AC27" s="11" t="n">
         <v>875.8200000000001</v>
       </c>
-      <c r="Y27" s="11" t="n">
+      <c r="AD27" s="11" t="n">
         <v>63.64</v>
       </c>
-      <c r="Z27" s="10" t="inlineStr">
+      <c r="AE27" s="10" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA27" s="10" t="inlineStr">
+      <c r="AF27" s="10" t="inlineStr">
         <is>
           <t>电子测量仪器和半导体测试设备的研发、制造、销售及服务</t>
         </is>
       </c>
-      <c r="AB27" s="10" t="inlineStr">
+      <c r="AG27" s="10" t="inlineStr">
         <is>
           <t>苏州联讯仪器股份有限公司</t>
         </is>
@@ -3415,22 +3848,39 @@
         <v>62.4</v>
       </c>
       <c r="X28" s="6" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="Y28" s="6" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="Z28" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="AA28" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB28" s="6" t="n">
+        <v>59.34</v>
+      </c>
+      <c r="AC28" s="6" t="n">
         <v>348.6</v>
       </c>
-      <c r="Y28" s="6" t="n">
+      <c r="AD28" s="6" t="n">
         <v>22.7</v>
       </c>
-      <c r="Z28" s="5" t="inlineStr">
+      <c r="AE28" s="5" t="inlineStr">
         <is>
           <t>国泰海通证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA28" s="5" t="inlineStr">
+      <c r="AF28" s="5" t="inlineStr">
         <is>
           <t>专注于物料自动配料、分散乳化、混合搅拌等物料自动化处理领域,提供专业的物料智能处理系统整体解决方案</t>
         </is>
       </c>
-      <c r="AB28" s="5" t="inlineStr">
+      <c r="AG28" s="5" t="inlineStr">
         <is>
           <t>无锡理奇智能装备股份有限公司</t>
         </is>
@@ -3523,22 +3973,39 @@
         <v>97.5</v>
       </c>
       <c r="X29" s="11" t="n">
+        <v>107.98</v>
+      </c>
+      <c r="Y29" s="11" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="Z29" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="AA29" s="11" t="n">
+        <v>122.22</v>
+      </c>
+      <c r="AB29" s="11" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="AC29" s="11" t="n">
         <v>633.08</v>
       </c>
-      <c r="Y29" s="11" t="n">
+      <c r="AD29" s="11" t="n">
         <v>26.02</v>
       </c>
-      <c r="Z29" s="10" t="inlineStr">
+      <c r="AE29" s="10" t="inlineStr">
         <is>
           <t>中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA29" s="10" t="inlineStr">
+      <c r="AF29" s="10" t="inlineStr">
         <is>
           <t>软磁铁氧体磁粉的研发、生产和销售,并沿产业链发展软磁铁氧体磁心、电子元器件和电源等产品</t>
         </is>
       </c>
-      <c r="AB29" s="10" t="inlineStr">
+      <c r="AG29" s="10" t="inlineStr">
         <is>
           <t>山东春光科技集团股份有限公司</t>
         </is>
@@ -3631,22 +4098,39 @@
         <v>91.84</v>
       </c>
       <c r="X30" s="6" t="n">
+        <v>110.28</v>
+      </c>
+      <c r="Y30" s="6" t="n">
+        <v>68.75</v>
+      </c>
+      <c r="Z30" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="AA30" s="6" t="n">
+        <v>99</v>
+      </c>
+      <c r="AB30" s="6" t="n">
+        <v>76.06</v>
+      </c>
+      <c r="AC30" s="6" t="n">
         <v>562.63</v>
       </c>
-      <c r="Y30" s="6" t="n">
+      <c r="AD30" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="Z30" s="5" t="inlineStr">
+      <c r="AE30" s="5" t="inlineStr">
         <is>
           <t>西南证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA30" s="5" t="inlineStr">
+      <c r="AF30" s="5" t="inlineStr">
         <is>
           <t>锆类产品、特种尼龙产品、精细化工产品的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB30" s="5" t="inlineStr">
+      <c r="AG30" s="5" t="inlineStr">
         <is>
           <t>长裕控股集团股份有限公司</t>
         </is>
@@ -3739,22 +4223,39 @@
         <v>120.67</v>
       </c>
       <c r="X31" s="11" t="n">
+        <v>150</v>
+      </c>
+      <c r="Y31" s="11" t="n">
+        <v>120</v>
+      </c>
+      <c r="Z31" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="AA31" s="11" t="n">
+        <v>107</v>
+      </c>
+      <c r="AB31" s="11" t="n">
+        <v>91</v>
+      </c>
+      <c r="AC31" s="11" t="n">
         <v>297.2</v>
       </c>
-      <c r="Y31" s="11" t="n">
+      <c r="AD31" s="11" t="n">
         <v>25.36</v>
       </c>
-      <c r="Z31" s="10" t="inlineStr">
+      <c r="AE31" s="10" t="inlineStr">
         <is>
           <t>中泰证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA31" s="10" t="inlineStr">
+      <c r="AF31" s="10" t="inlineStr">
         <is>
           <t>硬连接、柔性连接、触头组件、叠层母排和CCS等系列化电连接产品以及同步分解器等产品的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB31" s="10" t="inlineStr">
+      <c r="AG31" s="10" t="inlineStr">
         <is>
           <t>北京维通利电气股份有限公司</t>
         </is>
@@ -3847,22 +4348,39 @@
         <v>67.12</v>
       </c>
       <c r="X32" s="6" t="n">
+        <v>82.88</v>
+      </c>
+      <c r="Y32" s="6" t="n">
+        <v>61.02</v>
+      </c>
+      <c r="Z32" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="AA32" s="6" t="n">
+        <v>71.98</v>
+      </c>
+      <c r="AB32" s="6" t="n">
+        <v>61.05</v>
+      </c>
+      <c r="AC32" s="6" t="n">
         <v>146.86</v>
       </c>
-      <c r="Y32" s="6" t="n">
+      <c r="AD32" s="6" t="n">
         <v>23.4</v>
       </c>
-      <c r="Z32" s="5" t="inlineStr">
+      <c r="AE32" s="5" t="inlineStr">
         <is>
           <t>招商证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA32" s="5" t="inlineStr">
+      <c r="AF32" s="5" t="inlineStr">
         <is>
           <t>为汽车整车厂商提供汽车传输系统、连接系统、智能控制等解决方案,主营汽车线束、汽车连接器、汽车电子等汽车零部件产品的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB32" s="5" t="inlineStr">
+      <c r="AG32" s="5" t="inlineStr">
         <is>
           <t>天海汽车电子集团股份有限公司</t>
         </is>
@@ -3955,22 +4473,39 @@
         <v>111.8</v>
       </c>
       <c r="X33" s="11" t="n">
+        <v>161</v>
+      </c>
+      <c r="Y33" s="11" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="Z33" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="AA33" s="11" t="n">
+        <v>105.98</v>
+      </c>
+      <c r="AB33" s="11" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="AC33" s="11" t="n">
         <v>109.91</v>
       </c>
-      <c r="Y33" s="11" t="n">
+      <c r="AD33" s="11" t="n">
         <v>21.04</v>
       </c>
-      <c r="Z33" s="10" t="inlineStr">
+      <c r="AE33" s="10" t="inlineStr">
         <is>
           <t>财通证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA33" s="10" t="inlineStr">
+      <c r="AF33" s="10" t="inlineStr">
         <is>
           <t>深耕制冷领域,是一家以制冷设备的研发、生产及销售为核心业务的国家级高新技术企业</t>
         </is>
       </c>
-      <c r="AB33" s="10" t="inlineStr">
+      <c r="AG33" s="10" t="inlineStr">
         <is>
           <t>宁波惠康工业科技股份有限公司</t>
         </is>
@@ -4063,22 +4598,39 @@
         <v>127.68</v>
       </c>
       <c r="X34" s="6" t="n">
+        <v>140.91</v>
+      </c>
+      <c r="Y34" s="6" t="n">
+        <v>87.7</v>
+      </c>
+      <c r="Z34" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="AA34" s="6" t="n">
+        <v>112</v>
+      </c>
+      <c r="AB34" s="6" t="n">
+        <v>98.75</v>
+      </c>
+      <c r="AC34" s="6" t="n">
         <v>710.15</v>
       </c>
-      <c r="Y34" s="6" t="n">
+      <c r="AD34" s="6" t="n">
         <v>29.72</v>
       </c>
-      <c r="Z34" s="5" t="inlineStr">
+      <c r="AE34" s="5" t="inlineStr">
         <is>
           <t>广发证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA34" s="5" t="inlineStr">
+      <c r="AF34" s="5" t="inlineStr">
         <is>
           <t>BOPP电工膜研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB34" s="5" t="inlineStr">
+      <c r="AG34" s="5" t="inlineStr">
         <is>
           <t>泉州嘉德利电子材料股份公司</t>
         </is>
@@ -4171,22 +4723,39 @@
         <v>659.99</v>
       </c>
       <c r="X35" s="11" t="n">
+        <v>688.88</v>
+      </c>
+      <c r="Y35" s="11" t="n">
+        <v>522</v>
+      </c>
+      <c r="Z35" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="AA35" s="11" t="n">
+        <v>659.75</v>
+      </c>
+      <c r="AB35" s="11" t="n">
+        <v>550.99</v>
+      </c>
+      <c r="AC35" s="11" t="n">
         <v>1510.52</v>
       </c>
-      <c r="Y35" s="11" t="n">
+      <c r="AD35" s="11" t="n">
         <v>44.22</v>
       </c>
-      <c r="Z35" s="10" t="inlineStr">
+      <c r="AE35" s="10" t="inlineStr">
         <is>
           <t>国泰海通证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA35" s="10" t="inlineStr">
+      <c r="AF35" s="10" t="inlineStr">
         <is>
           <t>特种光纤的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB35" s="10" t="inlineStr">
+      <c r="AG35" s="10" t="inlineStr">
         <is>
           <t>武汉长进光子技术股份有限公司</t>
         </is>
@@ -4279,22 +4848,39 @@
         <v>51.3</v>
       </c>
       <c r="X36" s="6" t="n">
+        <v>63.65</v>
+      </c>
+      <c r="Y36" s="6" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="Z36" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="AA36" s="6" t="n">
+        <v>56.55</v>
+      </c>
+      <c r="AB36" s="6" t="n">
+        <v>49.96</v>
+      </c>
+      <c r="AC36" s="6" t="n">
         <v>624.58</v>
       </c>
-      <c r="Y36" s="6" t="n">
+      <c r="AD36" s="6" t="n">
         <v>29.97</v>
       </c>
-      <c r="Z36" s="5" t="inlineStr">
+      <c r="AE36" s="5" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA36" s="5" t="inlineStr">
+      <c r="AF36" s="5" t="inlineStr">
         <is>
           <t>公司主要面向新能源产业提供安全、可靠、高效、稳定且更具经济性的新型储能电池管理系统相关产品</t>
         </is>
       </c>
-      <c r="AB36" s="5" t="inlineStr">
+      <c r="AG36" s="5" t="inlineStr">
         <is>
           <t>杭州高特电子设备股份有限公司</t>
         </is>
@@ -4387,22 +4973,39 @@
         <v>585</v>
       </c>
       <c r="X37" s="11" t="n">
+        <v>589</v>
+      </c>
+      <c r="Y37" s="11" t="n">
+        <v>388.66</v>
+      </c>
+      <c r="Z37" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="AA37" s="11" t="n">
+        <v>619.97</v>
+      </c>
+      <c r="AB37" s="11" t="n">
+        <v>530</v>
+      </c>
+      <c r="AC37" s="11" t="n">
         <v>1212.84</v>
       </c>
-      <c r="Y37" s="11" t="n">
+      <c r="AD37" s="11" t="n">
         <v>31.31</v>
       </c>
-      <c r="Z37" s="10" t="inlineStr">
+      <c r="AE37" s="10" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA37" s="10" t="inlineStr">
+      <c r="AF37" s="10" t="inlineStr">
         <is>
           <t>为集成电路及显示面板行业客户提供制造设备真空腔体内参与工艺反应的零部件及其表面处理解决方案</t>
         </is>
       </c>
-      <c r="AB37" s="10" t="inlineStr">
+      <c r="AG37" s="10" t="inlineStr">
         <is>
           <t>重庆臻宝科技股份有限公司</t>
         </is>
@@ -4495,22 +5098,39 @@
         <v>42</v>
       </c>
       <c r="X38" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="Y38" s="6" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="Z38" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="AA38" s="6" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="AB38" s="6" t="n">
+        <v>33.66</v>
+      </c>
+      <c r="AC38" s="6" t="n">
         <v>315.02</v>
       </c>
-      <c r="Y38" s="6" t="n">
+      <c r="AD38" s="6" t="n">
         <v>25.45</v>
       </c>
-      <c r="Z38" s="5" t="inlineStr">
+      <c r="AE38" s="5" t="inlineStr">
         <is>
           <t>中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA38" s="5" t="inlineStr">
+      <c r="AF38" s="5" t="inlineStr">
         <is>
           <t>半导体显示面板等核心显示器件以及智能显示终端的研发、制造和销售</t>
         </is>
       </c>
-      <c r="AB38" s="5" t="inlineStr">
+      <c r="AG38" s="5" t="inlineStr">
         <is>
           <t>惠科股份有限公司</t>
         </is>
@@ -4603,22 +5223,39 @@
         <v>23.95</v>
       </c>
       <c r="X39" s="11" t="n">
+        <v>30.16</v>
+      </c>
+      <c r="Y39" s="11" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="Z39" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="AA39" s="11" t="n">
+        <v>23.38</v>
+      </c>
+      <c r="AB39" s="11" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="AC39" s="11" t="n">
         <v>136.89</v>
       </c>
-      <c r="Y39" s="11" t="n">
+      <c r="AD39" s="11" t="n">
         <v>21.99</v>
       </c>
-      <c r="Z39" s="10" t="inlineStr">
+      <c r="AE39" s="10" t="inlineStr">
         <is>
           <t>中信证券股份有限公司,中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA39" s="10" t="inlineStr">
+      <c r="AF39" s="10" t="inlineStr">
         <is>
           <t>投资、开发、运营和管理风力、太阳能发电站</t>
         </is>
       </c>
-      <c r="AB39" s="10" t="inlineStr">
+      <c r="AG39" s="10" t="inlineStr">
         <is>
           <t>华润新能源控股有限公司</t>
         </is>
@@ -4711,22 +5348,39 @@
         <v>216.7</v>
       </c>
       <c r="X40" s="6" t="n">
+        <v>264.42</v>
+      </c>
+      <c r="Y40" s="6" t="n">
+        <v>203.4</v>
+      </c>
+      <c r="Z40" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AA40" s="6" t="n">
+        <v>235.99</v>
+      </c>
+      <c r="AB40" s="6" t="n">
+        <v>206.98</v>
+      </c>
+      <c r="AC40" s="6" t="n">
         <v>858.85</v>
       </c>
-      <c r="Y40" s="6" t="n">
+      <c r="AD40" s="6" t="n">
         <v>44.82</v>
       </c>
-      <c r="Z40" s="5" t="inlineStr">
+      <c r="AE40" s="5" t="inlineStr">
         <is>
           <t>中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA40" s="5" t="inlineStr">
+      <c r="AF40" s="5" t="inlineStr">
         <is>
           <t>半导体及激光设备精密零部件的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB40" s="5" t="inlineStr">
+      <c r="AG40" s="5" t="inlineStr">
         <is>
           <t>托伦斯精密制造(江苏)股份有限公司</t>
         </is>
@@ -4819,20 +5473,37 @@
         <v>45.1</v>
       </c>
       <c r="X41" s="11" t="n">
+        <v>52.52</v>
+      </c>
+      <c r="Y41" s="11" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="Z41" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="AA41" s="11" t="n">
+        <v>43.47</v>
+      </c>
+      <c r="AB41" s="11" t="n">
+        <v>32.57</v>
+      </c>
+      <c r="AC41" s="11" t="n">
         <v>211.89</v>
       </c>
-      <c r="Y41" s="10" t="n"/>
-      <c r="Z41" s="10" t="inlineStr">
+      <c r="AD41" s="10" t="n"/>
+      <c r="AE41" s="10" t="inlineStr">
         <is>
           <t>华泰联合证券有限责任公司</t>
         </is>
       </c>
-      <c r="AA41" s="10" t="inlineStr">
+      <c r="AF41" s="10" t="inlineStr">
         <is>
           <t>全人源抗体药物的开发、生产和销售</t>
         </is>
       </c>
-      <c r="AB41" s="10" t="inlineStr">
+      <c r="AG41" s="10" t="inlineStr">
         <is>
           <t>珠海泰诺麦博制药股份有限公司</t>
         </is>
@@ -4925,22 +5596,39 @@
         <v>49</v>
       </c>
       <c r="X42" s="6" t="n">
+        <v>55.03</v>
+      </c>
+      <c r="Y42" s="6" t="n">
+        <v>38.11</v>
+      </c>
+      <c r="Z42" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="AA42" s="6" t="n">
+        <v>49.74</v>
+      </c>
+      <c r="AB42" s="6" t="n">
+        <v>45.21</v>
+      </c>
+      <c r="AC42" s="6" t="n">
         <v>465.82</v>
       </c>
-      <c r="Y42" s="6" t="n">
+      <c r="AD42" s="6" t="n">
         <v>308.92</v>
       </c>
-      <c r="Z42" s="5" t="inlineStr">
+      <c r="AE42" s="5" t="inlineStr">
         <is>
           <t>中信建投证券股份有限公司,中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA42" s="5" t="inlineStr">
+      <c r="AF42" s="5" t="inlineStr">
         <is>
           <t>DRAM产品的研发、设计、生产及销售</t>
         </is>
       </c>
-      <c r="AB42" s="5" t="inlineStr">
+      <c r="AG42" s="5" t="inlineStr">
         <is>
           <t>长鑫科技集团股份有限公司</t>
         </is>
@@ -5033,22 +5721,39 @@
         <v>82.40000000000001</v>
       </c>
       <c r="X43" s="11" t="n">
+        <v>110</v>
+      </c>
+      <c r="Y43" s="11" t="n">
+        <v>81</v>
+      </c>
+      <c r="Z43" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="AA43" s="11" t="n">
+        <v>110</v>
+      </c>
+      <c r="AB43" s="11" t="n">
+        <v>85.28</v>
+      </c>
+      <c r="AC43" s="11" t="n">
         <v>145.38</v>
       </c>
-      <c r="Y43" s="11" t="n">
+      <c r="AD43" s="11" t="n">
         <v>17.17</v>
       </c>
-      <c r="Z43" s="10" t="inlineStr">
+      <c r="AE43" s="10" t="inlineStr">
         <is>
           <t>华泰联合证券有限责任公司</t>
         </is>
       </c>
-      <c r="AA43" s="10" t="inlineStr">
+      <c r="AF43" s="10" t="inlineStr">
         <is>
           <t>孔加工刀具中钻削刀具产品的研发、生产和销售业务</t>
         </is>
       </c>
-      <c r="AB43" s="10" t="inlineStr">
+      <c r="AG43" s="10" t="inlineStr">
         <is>
           <t>浙江欣兴工具股份有限公司</t>
         </is>
@@ -5141,22 +5846,39 @@
         <v>208.01</v>
       </c>
       <c r="X44" s="6" t="n">
+        <v>234.5</v>
+      </c>
+      <c r="Y44" s="6" t="n">
+        <v>188.99</v>
+      </c>
+      <c r="Z44" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="AA44" s="6" t="n">
+        <v>209.68</v>
+      </c>
+      <c r="AB44" s="6" t="n">
+        <v>190.88</v>
+      </c>
+      <c r="AC44" s="6" t="n">
         <v>146.28</v>
       </c>
-      <c r="Y44" s="6" t="n">
+      <c r="AD44" s="6" t="n">
         <v>38.19</v>
       </c>
-      <c r="Z44" s="5" t="inlineStr">
+      <c r="AE44" s="5" t="inlineStr">
         <is>
           <t>国泰海通证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA44" s="5" t="inlineStr">
+      <c r="AF44" s="5" t="inlineStr">
         <is>
           <t>公司为业内领先、具有行业变革意义的电子产业基础设施综合服务提供商,为客户提供覆盖EDA/CAM工业软件、印制电路板制造、电子元器件购销及电子装联等全产业链一体化服务</t>
         </is>
       </c>
-      <c r="AB44" s="5" t="inlineStr">
+      <c r="AG44" s="5" t="inlineStr">
         <is>
           <t>深圳嘉立创科技集团股份有限公司</t>
         </is>
@@ -5249,22 +5971,39 @@
         <v>37.49</v>
       </c>
       <c r="X45" s="11" t="n">
+        <v>45.45</v>
+      </c>
+      <c r="Y45" s="11" t="n">
+        <v>36.89</v>
+      </c>
+      <c r="Z45" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AA45" s="11" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="AB45" s="11" t="n">
+        <v>30.67</v>
+      </c>
+      <c r="AC45" s="11" t="n">
         <v>114.72</v>
       </c>
-      <c r="Y45" s="11" t="n">
+      <c r="AD45" s="11" t="n">
         <v>19.25</v>
       </c>
-      <c r="Z45" s="10" t="inlineStr">
+      <c r="AE45" s="10" t="inlineStr">
         <is>
           <t>中泰证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA45" s="10" t="inlineStr">
+      <c r="AF45" s="10" t="inlineStr">
         <is>
           <t>从事自行车、电助力自行车、共享单车等产品及其关键零部件的研发、设计、生产与销售业务</t>
         </is>
       </c>
-      <c r="AB45" s="10" t="inlineStr">
+      <c r="AG45" s="10" t="inlineStr">
         <is>
           <t>天津富士达自行车工业股份有限公司</t>
         </is>
@@ -5357,22 +6096,39 @@
         <v>116.52</v>
       </c>
       <c r="X46" s="6" t="n">
+        <v>129.9</v>
+      </c>
+      <c r="Y46" s="6" t="n">
+        <v>106.88</v>
+      </c>
+      <c r="Z46" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AA46" s="6" t="n">
+        <v>115.99</v>
+      </c>
+      <c r="AB46" s="6" t="n">
+        <v>103.02</v>
+      </c>
+      <c r="AC46" s="6" t="n">
         <v>396.89</v>
       </c>
-      <c r="Y46" s="6" t="n">
+      <c r="AD46" s="6" t="n">
         <v>44.23</v>
       </c>
-      <c r="Z46" s="5" t="inlineStr">
+      <c r="AE46" s="5" t="inlineStr">
         <is>
           <t>华泰联合证券有限责任公司</t>
         </is>
       </c>
-      <c r="AA46" s="5" t="inlineStr">
+      <c r="AF46" s="5" t="inlineStr">
         <is>
           <t>高可靠模拟芯片及微模块产品的研发设计、测试及销售</t>
         </is>
       </c>
-      <c r="AB46" s="5" t="inlineStr">
+      <c r="AG46" s="5" t="inlineStr">
         <is>
           <t>江苏展芯半导体技术股份有限公司</t>
         </is>
@@ -5465,22 +6221,39 @@
         <v>503</v>
       </c>
       <c r="X47" s="11" t="n">
+        <v>554.73</v>
+      </c>
+      <c r="Y47" s="11" t="n">
+        <v>420</v>
+      </c>
+      <c r="Z47" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="AA47" s="11" t="n">
+        <v>524.4400000000001</v>
+      </c>
+      <c r="AB47" s="11" t="n">
+        <v>491</v>
+      </c>
+      <c r="AC47" s="11" t="n">
         <v>662.24</v>
       </c>
-      <c r="Y47" s="11" t="n">
+      <c r="AD47" s="11" t="n">
         <v>36.38</v>
       </c>
-      <c r="Z47" s="10" t="inlineStr">
+      <c r="AE47" s="10" t="inlineStr">
         <is>
           <t>华泰联合证券有限责任公司</t>
         </is>
       </c>
-      <c r="AA47" s="10" t="inlineStr">
+      <c r="AF47" s="10" t="inlineStr">
         <is>
           <t>主要从事半导体设备特殊涂层零部件和精密光学器件的研发、生产和销售。</t>
         </is>
       </c>
-      <c r="AB47" s="10" t="inlineStr">
+      <c r="AG47" s="10" t="inlineStr">
         <is>
           <t>成都超纯应用材料股份有限公司</t>
         </is>
@@ -5573,20 +6346,37 @@
         <v>110.23</v>
       </c>
       <c r="X48" s="6" t="n">
+        <v>118</v>
+      </c>
+      <c r="Y48" s="6" t="n">
+        <v>97.79000000000001</v>
+      </c>
+      <c r="Z48" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="AA48" s="6" t="n">
+        <v>124</v>
+      </c>
+      <c r="AB48" s="6" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="AC48" s="6" t="n">
         <v>419.46</v>
       </c>
-      <c r="Y48" s="5" t="n"/>
-      <c r="Z48" s="5" t="inlineStr">
+      <c r="AD48" s="5" t="n"/>
+      <c r="AE48" s="5" t="inlineStr">
         <is>
           <t>华泰联合证券有限责任公司</t>
         </is>
       </c>
-      <c r="AA48" s="5" t="inlineStr">
+      <c r="AF48" s="5" t="inlineStr">
         <is>
           <t>专注于高端科学仪器的研发,面向量子科技、材料科学、化学化工、生物医药、先进制造等多个领域,向全球范围内的高校及科研院所、企业提供科技前沿探索所需的高端科学仪器装备、以增强型量子传感器为代表的核心关键器件以及解决方案</t>
         </is>
       </c>
-      <c r="AB48" s="5" t="inlineStr">
+      <c r="AG48" s="5" t="inlineStr">
         <is>
           <t>国仪量子技术(合肥)股份有限公司</t>
         </is>
@@ -5679,22 +6469,39 @@
         <v>1152</v>
       </c>
       <c r="X49" s="11" t="n">
+        <v>1300</v>
+      </c>
+      <c r="Y49" s="11" t="n">
+        <v>1100</v>
+      </c>
+      <c r="Z49" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="AA49" s="11" t="n">
+        <v>1079</v>
+      </c>
+      <c r="AB49" s="11" t="n">
+        <v>940</v>
+      </c>
+      <c r="AC49" s="11" t="n">
         <v>516.4400000000001</v>
       </c>
-      <c r="Y49" s="11" t="n">
+      <c r="AD49" s="11" t="n">
         <v>49.42</v>
       </c>
-      <c r="Z49" s="10" t="inlineStr">
+      <c r="AE49" s="10" t="inlineStr">
         <is>
           <t>中信建投证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA49" s="10" t="inlineStr">
+      <c r="AF49" s="10" t="inlineStr">
         <is>
           <t>精准激光器的研发、生产与销售</t>
         </is>
       </c>
-      <c r="AB49" s="10" t="inlineStr">
+      <c r="AG49" s="10" t="inlineStr">
         <is>
           <t>上海频准激光科技股份有限公司</t>
         </is>
@@ -5787,22 +6594,39 @@
         <v>845</v>
       </c>
       <c r="X50" s="6" t="n">
+        <v>1100</v>
+      </c>
+      <c r="Y50" s="6" t="n">
+        <v>800.08</v>
+      </c>
+      <c r="Z50" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="AA50" s="6" t="n">
+        <v>790</v>
+      </c>
+      <c r="AB50" s="6" t="n">
+        <v>685.01</v>
+      </c>
+      <c r="AC50" s="6" t="n">
         <v>460.34</v>
       </c>
-      <c r="Y50" s="6" t="n">
+      <c r="AD50" s="6" t="n">
         <v>219.23</v>
       </c>
-      <c r="Z50" s="5" t="inlineStr">
+      <c r="AE50" s="5" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA50" s="5" t="inlineStr">
+      <c r="AF50" s="5" t="inlineStr">
         <is>
           <t>高性能通用人形机器人、四足机器人、机器人组件及具身智能模型的研发、生产和销售业务</t>
         </is>
       </c>
-      <c r="AB50" s="5" t="inlineStr">
+      <c r="AG50" s="5" t="inlineStr">
         <is>
           <t>宇树科技股份有限公司</t>
         </is>
@@ -5895,22 +6719,39 @@
         <v>32.49</v>
       </c>
       <c r="X51" s="11" t="n">
+        <v>43.79</v>
+      </c>
+      <c r="Y51" s="11" t="n">
+        <v>31.95</v>
+      </c>
+      <c r="Z51" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="AA51" s="11" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="AB51" s="11" t="n">
+        <v>26.57</v>
+      </c>
+      <c r="AC51" s="11" t="n">
         <v>282.24</v>
       </c>
-      <c r="Y51" s="11" t="n">
+      <c r="AD51" s="11" t="n">
         <v>27.56</v>
       </c>
-      <c r="Z51" s="10" t="inlineStr">
+      <c r="AE51" s="10" t="inlineStr">
         <is>
           <t>中国国际金融股份有限公司</t>
         </is>
       </c>
-      <c r="AA51" s="10" t="inlineStr">
+      <c r="AF51" s="10" t="inlineStr">
         <is>
           <t>新能源电驱动系统的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB51" s="10" t="inlineStr">
+      <c r="AG51" s="10" t="inlineStr">
         <is>
           <t>苏州绿控传动科技股份有限公司</t>
         </is>
@@ -5995,20 +6836,25 @@
       <c r="V52" s="15" t="n"/>
       <c r="W52" s="15" t="n"/>
       <c r="X52" s="15" t="n"/>
-      <c r="Y52" s="16" t="n">
+      <c r="Y52" s="15" t="n"/>
+      <c r="Z52" s="15" t="n"/>
+      <c r="AA52" s="15" t="n"/>
+      <c r="AB52" s="15" t="n"/>
+      <c r="AC52" s="15" t="n"/>
+      <c r="AD52" s="16" t="n">
         <v>48.33</v>
       </c>
-      <c r="Z52" s="15" t="inlineStr">
+      <c r="AE52" s="15" t="inlineStr">
         <is>
           <t>国泰海通证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA52" s="15" t="inlineStr">
+      <c r="AF52" s="15" t="inlineStr">
         <is>
           <t>精密流体控制领域中关键控制部件及相关设备的研发、生产与销售</t>
         </is>
       </c>
-      <c r="AB52" s="15" t="inlineStr">
+      <c r="AG52" s="15" t="inlineStr">
         <is>
           <t>江苏高凯精密流体技术股份有限公司</t>
         </is>
@@ -6079,7 +6925,7 @@
         <v>2306.15</v>
       </c>
       <c r="R53" s="18" t="n">
-        <v>2.7904</v>
+        <v>5.3229</v>
       </c>
       <c r="S53" s="18" t="n">
         <v>31.7867</v>
@@ -6089,20 +6935,25 @@
       <c r="V53" s="15" t="n"/>
       <c r="W53" s="15" t="n"/>
       <c r="X53" s="15" t="n"/>
-      <c r="Y53" s="16" t="n">
+      <c r="Y53" s="15" t="n"/>
+      <c r="Z53" s="15" t="n"/>
+      <c r="AA53" s="15" t="n"/>
+      <c r="AB53" s="15" t="n"/>
+      <c r="AC53" s="15" t="n"/>
+      <c r="AD53" s="16" t="n">
         <v>27.39</v>
       </c>
-      <c r="Z53" s="15" t="inlineStr">
+      <c r="AE53" s="15" t="inlineStr">
         <is>
           <t>国信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA53" s="15" t="inlineStr">
+      <c r="AF53" s="15" t="inlineStr">
         <is>
           <t>电子材料和化工新材料的研发、生产与销售</t>
         </is>
       </c>
-      <c r="AB53" s="15" t="inlineStr">
+      <c r="AG53" s="15" t="inlineStr">
         <is>
           <t>苏州市贝特利高分子材料股份有限公司</t>
         </is>
@@ -6181,20 +7032,25 @@
       <c r="V54" s="15" t="n"/>
       <c r="W54" s="15" t="n"/>
       <c r="X54" s="15" t="n"/>
-      <c r="Y54" s="16" t="n">
+      <c r="Y54" s="15" t="n"/>
+      <c r="Z54" s="15" t="n"/>
+      <c r="AA54" s="15" t="n"/>
+      <c r="AB54" s="15" t="n"/>
+      <c r="AC54" s="15" t="n"/>
+      <c r="AD54" s="16" t="n">
         <v>19.8</v>
       </c>
-      <c r="Z54" s="15" t="inlineStr">
+      <c r="AE54" s="15" t="inlineStr">
         <is>
           <t>长江证券承销保荐有限公司</t>
         </is>
       </c>
-      <c r="AA54" s="15" t="inlineStr">
+      <c r="AF54" s="15" t="inlineStr">
         <is>
           <t>香料产品的研发、生产与销售业务</t>
         </is>
       </c>
-      <c r="AB54" s="15" t="inlineStr">
+      <c r="AG54" s="15" t="inlineStr">
         <is>
           <t>格林生物科技股份有限公司</t>
         </is>
@@ -6273,20 +7129,25 @@
       <c r="V55" s="15" t="n"/>
       <c r="W55" s="15" t="n"/>
       <c r="X55" s="15" t="n"/>
-      <c r="Y55" s="16" t="n">
+      <c r="Y55" s="15" t="n"/>
+      <c r="Z55" s="15" t="n"/>
+      <c r="AA55" s="15" t="n"/>
+      <c r="AB55" s="15" t="n"/>
+      <c r="AC55" s="15" t="n"/>
+      <c r="AD55" s="16" t="n">
         <v>13.81</v>
       </c>
-      <c r="Z55" s="15" t="inlineStr">
+      <c r="AE55" s="15" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA55" s="15" t="inlineStr">
+      <c r="AF55" s="15" t="inlineStr">
         <is>
           <t>铁矿石的采选、综合利用及铁精粉、钼精矿销售,石灰石的开采和销售</t>
         </is>
       </c>
-      <c r="AB55" s="15" t="inlineStr">
+      <c r="AG55" s="15" t="inlineStr">
         <is>
           <t>福建马坑矿业股份有限公司</t>
         </is>
@@ -6363,20 +7224,25 @@
       <c r="V56" s="15" t="n"/>
       <c r="W56" s="15" t="n"/>
       <c r="X56" s="15" t="n"/>
-      <c r="Y56" s="16" t="n">
+      <c r="Y56" s="15" t="n"/>
+      <c r="Z56" s="15" t="n"/>
+      <c r="AA56" s="15" t="n"/>
+      <c r="AB56" s="15" t="n"/>
+      <c r="AC56" s="15" t="n"/>
+      <c r="AD56" s="16" t="n">
         <v>22.67</v>
       </c>
-      <c r="Z56" s="15" t="inlineStr">
+      <c r="AE56" s="15" t="inlineStr">
         <is>
           <t>中信建投证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA56" s="15" t="inlineStr">
+      <c r="AF56" s="15" t="inlineStr">
         <is>
           <t>轴承及相关零部件的研发、生产和销售</t>
         </is>
       </c>
-      <c r="AB56" s="15" t="inlineStr">
+      <c r="AG56" s="15" t="inlineStr">
         <is>
           <t>洛阳轴承集团股份有限公司</t>
         </is>
@@ -6453,20 +7319,25 @@
       <c r="V57" s="15" t="n"/>
       <c r="W57" s="15" t="n"/>
       <c r="X57" s="15" t="n"/>
-      <c r="Y57" s="16" t="n">
+      <c r="Y57" s="15" t="n"/>
+      <c r="Z57" s="15" t="n"/>
+      <c r="AA57" s="15" t="n"/>
+      <c r="AB57" s="15" t="n"/>
+      <c r="AC57" s="15" t="n"/>
+      <c r="AD57" s="16" t="n">
         <v>21.43</v>
       </c>
-      <c r="Z57" s="15" t="inlineStr">
+      <c r="AE57" s="15" t="inlineStr">
         <is>
           <t>中信建投证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA57" s="15" t="inlineStr">
+      <c r="AF57" s="15" t="inlineStr">
         <is>
           <t>汽车热管理系统零部件制造,并拓展了汽车声学部件等业务</t>
         </is>
       </c>
-      <c r="AB57" s="15" t="inlineStr">
+      <c r="AG57" s="15" t="inlineStr">
         <is>
           <t>天博智能科技(山东)股份有限公司</t>
         </is>
@@ -6534,17 +7405,22 @@
       <c r="W58" s="15" t="n"/>
       <c r="X58" s="15" t="n"/>
       <c r="Y58" s="15" t="n"/>
-      <c r="Z58" s="15" t="inlineStr">
+      <c r="Z58" s="15" t="n"/>
+      <c r="AA58" s="15" t="n"/>
+      <c r="AB58" s="15" t="n"/>
+      <c r="AC58" s="15" t="n"/>
+      <c r="AD58" s="15" t="n"/>
+      <c r="AE58" s="15" t="inlineStr">
         <is>
           <t>国泰海通证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA58" s="15" t="inlineStr">
+      <c r="AF58" s="15" t="inlineStr">
         <is>
           <t>从事电子测量仪器研发、制造和销售</t>
         </is>
       </c>
-      <c r="AB58" s="15" t="inlineStr">
+      <c r="AG58" s="15" t="inlineStr">
         <is>
           <t>中电科思仪科技股份有限公司</t>
         </is>
@@ -6612,27 +7488,32 @@
       <c r="W59" s="15" t="n"/>
       <c r="X59" s="15" t="n"/>
       <c r="Y59" s="15" t="n"/>
-      <c r="Z59" s="15" t="inlineStr">
+      <c r="Z59" s="15" t="n"/>
+      <c r="AA59" s="15" t="n"/>
+      <c r="AB59" s="15" t="n"/>
+      <c r="AC59" s="15" t="n"/>
+      <c r="AD59" s="15" t="n"/>
+      <c r="AE59" s="15" t="inlineStr">
         <is>
           <t>中信证券股份有限公司</t>
         </is>
       </c>
-      <c r="AA59" s="15" t="inlineStr">
+      <c r="AF59" s="15" t="inlineStr">
         <is>
           <t>公司坚持原始创新、自主研发的技术路线,构筑长期可持续发展的核心竞争力和护城河。成立近8年来,公司自研迭代了四代架构5款云端AI芯片,构建了覆盖AI芯片、AI加速卡及模组、智算系统及集群和AI计算及编程软件平台的完整产品体系</t>
         </is>
       </c>
-      <c r="AB59" s="15" t="inlineStr">
+      <c r="AG59" s="15" t="inlineStr">
         <is>
           <t>上海燧原科技股份有限公司</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:AB59"/>
+  <autoFilter ref="A3:AG59"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:AB2"/>
-    <mergeCell ref="A1:AB1"/>
+    <mergeCell ref="A2:AG2"/>
+    <mergeCell ref="A1:AG1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>